<commit_message>
The luminosity is also calculated via (B-V)\
</commit_message>
<xml_diff>
--- a/tables/HMXBparameters.xlsx
+++ b/tables/HMXBparameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luukv\Documenten\NatuurSterrkenkundeMasterProject\CodeMP\MasterProject\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324B2E90-1DD4-4740-8EC6-DB5A52817319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFA27D5-A9FF-4A68-8D5A-E66B8C7BAB74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5D7EFD20-82E9-4387-B64B-74E2094689FE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
   <si>
     <t>2S0114+650</t>
   </si>
@@ -177,6 +177,45 @@
   </si>
   <si>
     <t>JHK_err</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>B_err</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>V_err</t>
+  </si>
+  <si>
+    <t>B_source</t>
+  </si>
+  <si>
+    <t>V_source</t>
+  </si>
+  <si>
+    <t>Tycho-2 </t>
+  </si>
+  <si>
+    <t>MC survey</t>
+  </si>
+  <si>
+    <t>2002yCat.2237....0D</t>
+  </si>
+  <si>
+    <t>Integral</t>
+  </si>
+  <si>
+    <t>2012yCat.1322....0Z</t>
+  </si>
+  <si>
+    <t>2014MNRAS.440.1626M</t>
+  </si>
+  <si>
+    <t>2015A&amp;A...574A..33R</t>
   </si>
 </sst>
 </file>
@@ -295,7 +334,251 @@
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -654,18 +937,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{92CB420E-405D-4566-9783-CE3C03E82CE3}" name="Tabel13" displayName="Tabel13" ref="A1:I16" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
-  <autoFilter ref="A1:I16" xr:uid="{92CB420E-405D-4566-9783-CE3C03E82CE3}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{3CDFCB5F-FC45-4284-B98B-6569A50499F1}" name="id" totalsRowLabel="Totaal" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{62D3F204-AEF7-43A9-B874-81735D76945A}" name="ST" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{8AA09B7A-CD50-481C-B71F-3707B0FEE3AD}" name="ST_ref" dataDxfId="11"/>
-    <tableColumn id="16" xr3:uid="{6E189503-68AD-41D0-89B7-F8BD4EFBCD13}" name="ruwe" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{24F2687F-2F36-4789-A274-A7BA379BB679}" name="J" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{E63669D6-EF94-4783-8FBA-9518CBF67162}" name="H" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{8C514BBF-8AE2-487A-B056-30A9A8F46585}" name="K" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{6AE7B876-5FE3-417F-AC5A-A25DFFEF608C}" name="JHK_ref" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{E8A67492-C113-44E4-9619-55E1A3E9A2BB}" name="JHK_err" dataDxfId="1" totalsRowDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{92CB420E-405D-4566-9783-CE3C03E82CE3}" name="Tabel13" displayName="Tabel13" ref="A1:O16" headerRowDxfId="28" dataDxfId="27" totalsRowDxfId="26">
+  <autoFilter ref="A1:O16" xr:uid="{92CB420E-405D-4566-9783-CE3C03E82CE3}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{3CDFCB5F-FC45-4284-B98B-6569A50499F1}" name="id" totalsRowLabel="Totaal" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{62D3F204-AEF7-43A9-B874-81735D76945A}" name="ST" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{8AA09B7A-CD50-481C-B71F-3707B0FEE3AD}" name="ST_ref" dataDxfId="23"/>
+    <tableColumn id="16" xr3:uid="{6E189503-68AD-41D0-89B7-F8BD4EFBCD13}" name="ruwe" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{24F2687F-2F36-4789-A274-A7BA379BB679}" name="J" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{E63669D6-EF94-4783-8FBA-9518CBF67162}" name="H" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{8C514BBF-8AE2-487A-B056-30A9A8F46585}" name="K" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{6AE7B876-5FE3-417F-AC5A-A25DFFEF608C}" name="JHK_ref" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{E8A67492-C113-44E4-9619-55E1A3E9A2BB}" name="JHK_err" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{1EC6AD36-0F8C-405B-A28B-ADF6A5245D1D}" name="B" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{0835DEFA-DDC0-494C-BF77-E378448E347D}" name="B_err" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{8A31223E-45E2-4F62-B853-B924425A1237}" name="B_source" dataDxfId="2" totalsRowDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{3002717A-F5EB-4CDD-B553-8A0BF3CBDCE8}" name="V" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{C372DDA1-9429-4DBE-96AF-350FBC6315C0}" name="V_err" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{594FA272-63E9-40E6-9EC3-EEB816BAEF6B}" name="V_source" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -968,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DE1212-5B01-4B9B-B604-F1E7439DEFE1}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -976,9 +1265,11 @@
     <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -1003,11 +1294,29 @@
       <c r="H1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
+      <c r="J1" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="M1" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="N1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:15">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1032,11 +1341,29 @@
       <c r="H2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I2" s="16">
+      <c r="I2" s="4">
         <v>0.03</v>
       </c>
+      <c r="J2" s="16">
+        <v>11.99</v>
+      </c>
+      <c r="K2" s="16">
+        <v>0.12</v>
+      </c>
+      <c r="L2" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" s="16">
+        <v>11.14</v>
+      </c>
+      <c r="N2" s="16">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="O2" s="16" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:15">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1061,11 +1388,25 @@
       <c r="H3" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I3" s="16">
+      <c r="I3" s="4">
         <v>0.03</v>
       </c>
+      <c r="J3" s="16">
+        <v>13</v>
+      </c>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M3" s="16">
+        <v>13.15</v>
+      </c>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:15">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1090,11 +1431,21 @@
       <c r="H4" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="16">
+      <c r="I4" s="4">
         <v>0.03</v>
       </c>
+      <c r="J4" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16">
+        <v>14</v>
+      </c>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:15">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -1119,11 +1470,25 @@
       <c r="H5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="16">
+      <c r="I5" s="4">
         <v>0.03</v>
       </c>
+      <c r="J5" s="16">
+        <v>7.37</v>
+      </c>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M5" s="16">
+        <v>6.87</v>
+      </c>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:15">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -1142,11 +1507,25 @@
       <c r="H6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="16">
+      <c r="I6" s="4">
         <v>0.03</v>
       </c>
+      <c r="J6" s="16">
+        <v>14.4</v>
+      </c>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16">
+        <v>12.27</v>
+      </c>
+      <c r="N6" s="16">
+        <v>0.08</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:15">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
@@ -1171,11 +1550,29 @@
       <c r="H7" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="4">
         <v>0.03</v>
       </c>
+      <c r="J7" s="16">
+        <v>12.481999999999999</v>
+      </c>
+      <c r="K7" s="16">
+        <v>0.04</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M7" s="16">
+        <v>10.803000000000001</v>
+      </c>
+      <c r="N7" s="16">
+        <v>0.04</v>
+      </c>
+      <c r="O7" s="16" t="s">
+        <v>57</v>
+      </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:15">
       <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
@@ -1200,11 +1597,23 @@
       <c r="H8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I8" s="16">
+      <c r="I8" s="4">
         <v>0.03</v>
       </c>
+      <c r="J8" s="16">
+        <v>16.3</v>
+      </c>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16">
+        <v>14.5</v>
+      </c>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:15">
       <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
@@ -1229,11 +1638,25 @@
       <c r="H9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="4">
         <v>0.03</v>
       </c>
+      <c r="J9" s="16">
+        <v>6.78</v>
+      </c>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M9" s="16">
+        <v>6.51</v>
+      </c>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:15">
       <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
@@ -1250,11 +1673,25 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
-      <c r="I10" s="16">
+      <c r="I10" s="4">
         <v>0.03</v>
       </c>
+      <c r="J10" s="16">
+        <v>19.41</v>
+      </c>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M10" s="16">
+        <v>16.350000000000001</v>
+      </c>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:15">
       <c r="A11" s="5" t="s">
         <v>9</v>
       </c>
@@ -1279,11 +1716,21 @@
       <c r="H11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I11" s="16">
+      <c r="I11" s="4">
         <v>0.03</v>
       </c>
+      <c r="J11" s="16">
+        <v>14.8</v>
+      </c>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16">
+        <v>14.5</v>
+      </c>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:15">
       <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
@@ -1308,11 +1755,25 @@
       <c r="H12" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="4">
         <v>0.03</v>
       </c>
+      <c r="J12" s="16">
+        <v>9.7200000000000006</v>
+      </c>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M12" s="16">
+        <v>8.91</v>
+      </c>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:15">
       <c r="A13" s="10" t="s">
         <v>17</v>
       </c>
@@ -1327,11 +1788,21 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
-      <c r="I13" s="16">
+      <c r="I13" s="4">
         <v>0.03</v>
       </c>
+      <c r="J13" s="16">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="N13" s="16"/>
+      <c r="O13" s="16"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:15">
       <c r="A14" s="5" t="s">
         <v>25</v>
       </c>
@@ -1354,11 +1825,27 @@
       <c r="H14" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="4">
         <v>0.03</v>
       </c>
+      <c r="J14" s="16">
+        <v>16.451000000000001</v>
+      </c>
+      <c r="K14" s="16">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M14" s="16">
+        <v>14.512</v>
+      </c>
+      <c r="N14" s="16">
+        <v>0.01</v>
+      </c>
+      <c r="O14" s="16"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:15">
       <c r="A15" s="5" t="s">
         <v>18</v>
       </c>
@@ -1381,11 +1868,17 @@
       <c r="H15" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="16">
+      <c r="I15" s="4">
         <v>0.03</v>
       </c>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:15">
       <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
@@ -1408,9 +1901,15 @@
       <c r="H16" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="4">
         <v>0.03</v>
       </c>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished model fit run
</commit_message>
<xml_diff>
--- a/tables/HMXBparameters.xlsx
+++ b/tables/HMXBparameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luukv\Documenten\NatuurSterrkenkundeMasterProject\CodeMP\MasterProject\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFA27D5-A9FF-4A68-8D5A-E66B8C7BAB74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3E554E-75A0-4EE7-A73A-787F592E5AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5D7EFD20-82E9-4387-B64B-74E2094689FE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
   <si>
     <t>2S0114+650</t>
   </si>
@@ -168,9 +168,6 @@
   </si>
   <si>
     <t>2MASS</t>
-  </si>
-  <si>
-    <t>E(B-V) from van der Meer et al. (2007)</t>
   </si>
   <si>
     <t>B0Ia</t>
@@ -287,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -324,12 +321,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -378,6 +369,106 @@
     <dxf>
       <font>
         <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibr  "/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -398,106 +489,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibr  "/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibr  "/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -951,9 +942,9 @@
     <tableColumn id="8" xr3:uid="{E8A67492-C113-44E4-9619-55E1A3E9A2BB}" name="JHK_err" dataDxfId="13" totalsRowDxfId="12"/>
     <tableColumn id="9" xr3:uid="{1EC6AD36-0F8C-405B-A28B-ADF6A5245D1D}" name="B" dataDxfId="11" totalsRowDxfId="10"/>
     <tableColumn id="10" xr3:uid="{0835DEFA-DDC0-494C-BF77-E378448E347D}" name="B_err" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{8A31223E-45E2-4F62-B853-B924425A1237}" name="B_source" dataDxfId="2" totalsRowDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{3002717A-F5EB-4CDD-B553-8A0BF3CBDCE8}" name="V" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{C372DDA1-9429-4DBE-96AF-350FBC6315C0}" name="V_err" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{8A31223E-45E2-4F62-B853-B924425A1237}" name="B_source" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{3002717A-F5EB-4CDD-B553-8A0BF3CBDCE8}" name="V" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{C372DDA1-9429-4DBE-96AF-350FBC6315C0}" name="V_err" dataDxfId="3" totalsRowDxfId="2"/>
     <tableColumn id="14" xr3:uid="{594FA272-63E9-40E6-9EC3-EEB816BAEF6B}" name="V_source" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1295,25 +1286,25 @@
         <v>42</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="K1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="L1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="N1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="M1" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="N1" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="O1" s="17" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -1344,23 +1335,23 @@
       <c r="I2" s="4">
         <v>0.03</v>
       </c>
-      <c r="J2" s="16">
+      <c r="J2" s="4">
         <v>11.99</v>
       </c>
-      <c r="K2" s="16">
+      <c r="K2" s="4">
         <v>0.12</v>
       </c>
-      <c r="L2" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="M2" s="16">
+      <c r="L2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="M2" s="4">
         <v>11.14</v>
       </c>
-      <c r="N2" s="16">
+      <c r="N2" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="O2" s="16" t="s">
-        <v>53</v>
+      <c r="O2" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -1391,19 +1382,19 @@
       <c r="I3" s="4">
         <v>0.03</v>
       </c>
-      <c r="J3" s="16">
+      <c r="J3" s="4">
         <v>13</v>
       </c>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="M3" s="16">
+      <c r="K3" s="4"/>
+      <c r="L3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="M3" s="4">
         <v>13.15</v>
       </c>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16" t="s">
-        <v>54</v>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -1434,16 +1425,16 @@
       <c r="I4" s="4">
         <v>0.03</v>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="4">
         <v>13.9</v>
       </c>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16">
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4">
         <v>14</v>
       </c>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="5" t="s">
@@ -1473,19 +1464,19 @@
       <c r="I5" s="4">
         <v>0.03</v>
       </c>
-      <c r="J5" s="16">
+      <c r="J5" s="4">
         <v>7.37</v>
       </c>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="M5" s="16">
+      <c r="K5" s="4"/>
+      <c r="L5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M5" s="4">
         <v>6.87</v>
       </c>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16" t="s">
-        <v>55</v>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -1501,28 +1492,34 @@
       <c r="D6" s="6">
         <v>1.0207037000000001</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="E6" s="12">
+        <v>10.736000000000001</v>
+      </c>
+      <c r="F6" s="12">
+        <v>10.311</v>
+      </c>
+      <c r="G6" s="12">
+        <v>10.093</v>
+      </c>
       <c r="H6" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I6" s="4">
         <v>0.03</v>
       </c>
-      <c r="J6" s="16">
+      <c r="J6" s="4">
         <v>14.4</v>
       </c>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16">
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4">
         <v>12.27</v>
       </c>
-      <c r="N6" s="16">
+      <c r="N6" s="4">
         <v>0.08</v>
       </c>
-      <c r="O6" s="16" t="s">
-        <v>56</v>
+      <c r="O6" s="4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -1553,23 +1550,23 @@
       <c r="I7" s="4">
         <v>0.03</v>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="4">
         <v>12.481999999999999</v>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="4">
         <v>0.04</v>
       </c>
-      <c r="L7" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="M7" s="16">
+      <c r="L7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" s="4">
         <v>10.803000000000001</v>
       </c>
-      <c r="N7" s="16">
+      <c r="N7" s="4">
         <v>0.04</v>
       </c>
-      <c r="O7" s="16" t="s">
-        <v>57</v>
+      <c r="O7" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -1577,7 +1574,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>37</v>
@@ -1600,17 +1597,17 @@
       <c r="I8" s="4">
         <v>0.03</v>
       </c>
-      <c r="J8" s="16">
+      <c r="J8" s="4">
         <v>16.3</v>
       </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16">
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4">
         <v>14.5</v>
       </c>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16" t="s">
-        <v>58</v>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -1641,19 +1638,19 @@
       <c r="I9" s="4">
         <v>0.03</v>
       </c>
-      <c r="J9" s="16">
+      <c r="J9" s="4">
         <v>6.78</v>
       </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="M9" s="16">
+      <c r="K9" s="4"/>
+      <c r="L9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M9" s="4">
         <v>6.51</v>
       </c>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16" t="s">
-        <v>55</v>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -1676,19 +1673,19 @@
       <c r="I10" s="4">
         <v>0.03</v>
       </c>
-      <c r="J10" s="16">
+      <c r="J10" s="4">
         <v>19.41</v>
       </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="M10" s="16">
+      <c r="K10" s="4"/>
+      <c r="L10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="M10" s="4">
         <v>16.350000000000001</v>
       </c>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16" t="s">
-        <v>59</v>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1719,16 +1716,16 @@
       <c r="I11" s="4">
         <v>0.03</v>
       </c>
-      <c r="J11" s="16">
+      <c r="J11" s="4">
         <v>14.8</v>
       </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16">
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4">
         <v>14.5</v>
       </c>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="5" t="s">
@@ -1758,19 +1755,19 @@
       <c r="I12" s="4">
         <v>0.03</v>
       </c>
-      <c r="J12" s="16">
+      <c r="J12" s="4">
         <v>9.7200000000000006</v>
       </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="M12" s="16">
+      <c r="K12" s="4"/>
+      <c r="L12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M12" s="4">
         <v>8.91</v>
       </c>
-      <c r="N12" s="16"/>
-      <c r="O12" s="16" t="s">
-        <v>55</v>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1791,16 +1788,16 @@
       <c r="I13" s="4">
         <v>0.03</v>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="4">
         <v>17.399999999999999</v>
       </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16">
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4">
         <v>16.399999999999999</v>
       </c>
-      <c r="N13" s="16"/>
-      <c r="O13" s="16"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="5" t="s">
@@ -1828,22 +1825,22 @@
       <c r="I14" s="4">
         <v>0.03</v>
       </c>
-      <c r="J14" s="16">
+      <c r="J14" s="4">
         <v>16.451000000000001</v>
       </c>
-      <c r="K14" s="16">
+      <c r="K14" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="L14" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="M14" s="16">
+      <c r="L14" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" s="4">
         <v>14.512</v>
       </c>
-      <c r="N14" s="16">
+      <c r="N14" s="4">
         <v>0.01</v>
       </c>
-      <c r="O14" s="16"/>
+      <c r="O14" s="4"/>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="5" t="s">
@@ -1871,12 +1868,12 @@
       <c r="I15" s="4">
         <v>0.03</v>
       </c>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-      <c r="O15" s="16"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="5" t="s">
@@ -1904,12 +1901,12 @@
       <c r="I16" s="4">
         <v>0.03</v>
       </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
-      <c r="O16" s="16"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Minor changes to luminosity.ipynb
</commit_message>
<xml_diff>
--- a/tables/HMXBparameters.xlsx
+++ b/tables/HMXBparameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luukv\Documenten\NatuurSterrkenkundeMasterProject\CodeMP\MasterProject\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3E554E-75A0-4EE7-A73A-787F592E5AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674FE1AE-E93C-4170-B2A6-601DEA3FB1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5D7EFD20-82E9-4387-B64B-74E2094689FE}"/>
   </bookViews>
@@ -1513,7 +1513,7 @@
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4">
-        <v>12.27</v>
+        <v>13.4</v>
       </c>
       <c r="N6" s="4">
         <v>0.08</v>

</xml_diff>